<commit_message>
feat(agent): standardize feature screening flow
</commit_message>
<xml_diff>
--- a/projects/2026-05-fujie-gcard-v1/reports/feature_screening_process.xlsx
+++ b/projects/2026-05-fujie-gcard-v1/reports/feature_screening_process.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Screening" sheetId="1" r:id="Rdec73521774e49ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Data" sheetId="2" r:id="R990264edea344698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Screening" sheetId="1" r:id="R8ee8618924804916"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Data" sheetId="2" r:id="R57ab0b3a42f34ba1"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>